<commit_message>
Uploaded updated time management, weekly blogs and project outline
</commit_message>
<xml_diff>
--- a/Config/Time Management.xlsx
+++ b/Config/Time Management.xlsx
@@ -1,29 +1,97 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\GIT Projects\MMP-RoverGame\Config\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7EDDE0-7C38-4497-BFAA-2492CDCFDFC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="6585" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Hours Worked</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Hours Owed</t>
+  </si>
+  <si>
+    <t>W/C</t>
+  </si>
+  <si>
+    <t>Total Owed Hours</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="22"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -49,13 +117,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -330,10 +444,243 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A2" s="4">
+        <v>45684</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1">
+        <f>30-B2</f>
+        <v>30</v>
+      </c>
+      <c r="E2" s="6">
+        <f>SUM(D2:D11)</f>
+        <v>283</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A3" s="4">
+        <v>45691</v>
+      </c>
+      <c r="B3" s="1">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1">
+        <f t="shared" ref="D3:D15" si="0">30-B3</f>
+        <v>13</v>
+      </c>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A4" s="4">
+        <v>45698</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A5" s="4">
+        <v>45705</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A6" s="4">
+        <v>45712</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A7" s="4">
+        <v>45719</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A8" s="4">
+        <v>45726</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A9" s="4">
+        <v>45733</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A10" s="4">
+        <v>45740</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A11" s="4">
+        <v>45747</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A12" s="4">
+        <v>45754</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A13" s="4">
+        <v>45761</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A14" s="4">
+        <v>45768</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
+      <c r="A15" s="4">
+        <v>45775</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2:C15">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>B2&lt;20</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>B2&gt;=30</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="7">
+      <formula>AND(B2&gt;=20, B2&lt;30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16:D1048576">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>B16&gt;=30</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>AND(B16&gt;=20, B16&lt;30)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Week 03 Push To Dev
My push for week 3. Refer to end of week notes for all content added.
</commit_message>
<xml_diff>
--- a/Config/Time Management.xlsx
+++ b/Config/Time Management.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\GIT Projects\MMP-RoverGame\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7EDDE0-7C38-4497-BFAA-2492CDCFDFC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAA5D5F-6A91-49C3-B8F4-F6983A83D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6585" yWindow="-16200" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7830" yWindow="-15060" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -477,7 +477,9 @@
       <c r="A2" s="4">
         <v>45684</v>
       </c>
-      <c r="B2" s="1"/>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1">
         <f>30-B2</f>
@@ -485,7 +487,7 @@
       </c>
       <c r="E2" s="6">
         <f>SUM(D2:D11)</f>
-        <v>283</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.65">
@@ -506,11 +508,13 @@
       <c r="A4" s="4">
         <v>45698</v>
       </c>
-      <c r="B4" s="1"/>
+      <c r="B4" s="1">
+        <v>17</v>
+      </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E4" s="1"/>
     </row>

</xml_diff>